<commit_message>
Model bus sections and couplers with generic section-aware routing
</commit_message>
<xml_diff>
--- a/samples/ss_krian12_gresik_ingest.xlsx
+++ b/samples/ss_krian12_gresik_ingest.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gardu_Induk_dan_Aset" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jalur_Transmisi" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Kerawanan_Detail" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kopel_Bus" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Kerawanan_Detail" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U55"/>
+  <dimension ref="A1:X55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,6 +616,21 @@
           <t>Longitude</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Seksi Bus</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Seksi Bus HV</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Seksi Bus LV</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1519,6 +1535,11 @@
           <t>150 kV</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Seksi 1/2: ID model; bay belum dipetakan; kopel OPEN per risiko #9</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -1537,6 +1558,11 @@
       <c r="R20" t="inlineStr">
         <is>
           <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>1;2</t>
         </is>
       </c>
     </row>
@@ -1936,6 +1962,11 @@
           <t>Jawa Timur</t>
         </is>
       </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>A;B</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2941,6 +2972,11 @@
       <c r="R51" t="inlineStr">
         <is>
           <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>A;B</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3221,6 +3257,21 @@
           <t>Sudut Pandang</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Seksi Dari</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Seksi Ke</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>No Sirkit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -4299,7 +4350,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
         </is>
       </c>
     </row>
@@ -4358,7 +4409,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
         </is>
       </c>
     </row>
@@ -4533,6 +4584,11 @@
           <t>Tidak</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -4808,6 +4864,11 @@
           <t>Tidak</t>
         </is>
       </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4867,6 +4928,11 @@
           <t>Tidak</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4921,6 +4987,11 @@
           <t>Tidak</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -5029,6 +5100,11 @@
           <t>Tidak</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -5815,6 +5891,11 @@
           <t>Tidak</t>
         </is>
       </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -5874,6 +5955,11 @@
           <t>Tidak</t>
         </is>
       </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -5989,7 +6075,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
         </is>
       </c>
     </row>
@@ -6048,7 +6134,12 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -6082,7 +6173,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -6108,6 +6199,16 @@
       <c r="P52" t="inlineStr">
         <is>
           <t>Tidak</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -6117,31 +6218,31 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SUTT Sampang - Pamekasan</t>
+          <t>SUTT Bangkalan - Sampang</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
+          <t>BKLAN</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
           <t>SAMPG</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>PKSAN</t>
-        </is>
-      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>150 kV</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -6159,14 +6260,24 @@
         </is>
       </c>
       <c r="N53" t="n">
+        <v>9</v>
+      </c>
+      <c r="O53" t="n">
         <v>10</v>
       </c>
-      <c r="O53" t="n">
-        <v>11</v>
-      </c>
       <c r="P53" t="inlineStr">
         <is>
           <t>Tidak</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -6174,19 +6285,24 @@
       <c r="A54" t="n">
         <v>53</v>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SUTT Pamekasan - Guluk-Guluk</t>
+          <t>SUTT Sampang - Pamekasan</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
+          <t>SAMPG</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
           <t>PKSAN</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>GULUK</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6204,7 +6320,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Sangat Rawan</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -6213,10 +6329,10 @@
         </is>
       </c>
       <c r="N54" t="n">
+        <v>10</v>
+      </c>
+      <c r="O54" t="n">
         <v>11</v>
-      </c>
-      <c r="O54" t="n">
-        <v>12</v>
       </c>
       <c r="P54" t="inlineStr">
         <is>
@@ -6230,17 +6346,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SUTT Guluk-Guluk - Sumenep</t>
+          <t>SUTT Pamekasan - Guluk-Guluk</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
+          <t>PKSAN</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
           <t>GULUK</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>SMNEP</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6267,12 +6383,66 @@
         </is>
       </c>
       <c r="N55" t="n">
+        <v>11</v>
+      </c>
+      <c r="O55" t="n">
         <v>12</v>
       </c>
-      <c r="O55" t="n">
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SUTT Guluk-Guluk - Sumenep</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GULUK</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SMNEP</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>2</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Jawa Timur</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>12</v>
+      </c>
+      <c r="O56" t="n">
         <v>13</v>
       </c>
-      <c r="P55" t="inlineStr">
+      <c r="P56" t="inlineStr">
         <is>
           <t>Tidak</t>
         </is>
@@ -6289,6 +6459,168 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kode GI</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID Kopel</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Seksi Dari</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Seksi Ke</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status Kopel</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>No Kerawanan</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Sudut Pandang</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RNKUT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>KOP_AB</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kopel Rungkut A-B; Gambar 5.3; splitting sesuai mitigasi #3. Posisi sumber buku, bukan telemetri.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BKLAN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>KOP_AB</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Kopel Bangkalan A-B dibuka; Tabel 5.1 #21 dan Gambar 5.3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SWHAN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KOP_12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Kopel Sawahan dibuka per #9; terminal belum dipetakan; 1/2 adalah ID model.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>